<commit_message>
Updated NOR_grids_kan10 model - 2026-06-24 17:45
</commit_message>
<xml_diff>
--- a/VerveStacks_NOR_grids_kan10/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_NOR_grids_kan10/ReportDefs_vervestacks.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_NOR_grids_kan10\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F4FE55B6-A737-4904-81D8-3DC020038202}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{F463AC5F-8A81-41DE-B531-CF8F029256F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3308" yWindow="3308" windowWidth="21600" windowHeight="12682" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ScenMap" sheetId="70" r:id="rId1"/>
@@ -23830,7 +23830,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{24AA394E-EA08-4372-AE02-B894E2A1EBF9}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0EE667C5-1807-4D3C-B90D-917CDF68EF4A}">
   <dimension ref="B9:H79"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -25248,7 +25248,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{619885B9-2164-42E9-82A5-2D999DBD1E05}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00CED21A-0944-493C-8094-A16F371208F2}">
   <dimension ref="B9:L79"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>